<commit_message>
260312 commit 测试github actions
</commit_message>
<xml_diff>
--- a/vessels/vessels_db.xlsx
+++ b/vessels/vessels_db.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Files\demo\capaStudy\vessels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A07FBEF-0C77-4E93-88C1-9C1B49898FEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BCDBBCB-7843-42E2-AE70-B1AFAD340F37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5130" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="vessels" sheetId="1" r:id="rId1"/>
@@ -40177,8 +40177,8 @@
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.06640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.1328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.86328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.46484375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15.75" x14ac:dyDescent="0.3">

</xml_diff>